<commit_message>
Add employee import template generation and update Excel import service for parent details handling
</commit_message>
<xml_diff>
--- a/frontend/public/template-karyawan.xlsx
+++ b/frontend/public/template-karyawan.xlsx
@@ -10,39 +10,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="B1" authorId="0">
-      <text>
-        <r>
-          <t>Mandatory. Unique Employee ID.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0">
-      <text>
-        <r>
-          <t>Mandatory. Full Name.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0">
-      <text>
-        <r>
-          <t>YYYY-MM-DD</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
   <si>
     <t>NOMOR INDUK KARYAWAN</t>
   </si>
@@ -354,6 +323,24 @@
   </si>
   <si>
     <t>KETERANGAN SAUDARA KANDUNG 4</t>
+  </si>
+  <si>
+    <t>NAMA SAUDARA KANDUNG 5</t>
+  </si>
+  <si>
+    <t>JENIS KELAMIN SAUDARA KANDUNG 5</t>
+  </si>
+  <si>
+    <t>TANGGAL LAHIR SAUDARA KANDUNG 5</t>
+  </si>
+  <si>
+    <t>PENDIDIKAN TERAKHIR SAUDARA KANDUNG 5</t>
+  </si>
+  <si>
+    <t>PEKERJAAN SAUDARA KANDUNG 5</t>
+  </si>
+  <si>
+    <t>KETERANGAN SAUDARA KANDUNG 5</t>
   </si>
   <si>
     <t>SIKLUS PEMBAYARAN</t>
@@ -481,20 +468,14 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2F75B5"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -511,8 +492,8 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -856,77 +837,133 @@
   <dimension ref="A1:EQ1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="35" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="6" width="15" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="4" width="18" customWidth="1"/>
+    <col min="5" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="20" customWidth="1"/>
-    <col min="15" max="20" width="15" customWidth="1"/>
-    <col min="21" max="21" width="40" customWidth="1"/>
-    <col min="22" max="23" width="20" customWidth="1"/>
-    <col min="24" max="27" width="15" customWidth="1"/>
-    <col min="28" max="28" width="10" customWidth="1"/>
-    <col min="29" max="29" width="20" customWidth="1"/>
-    <col min="30" max="30" width="40" customWidth="1"/>
-    <col min="31" max="34" width="20" customWidth="1"/>
-    <col min="35" max="35" width="30" customWidth="1"/>
-    <col min="36" max="36" width="20" customWidth="1"/>
-    <col min="37" max="37" width="10" customWidth="1"/>
-    <col min="38" max="38" width="15" customWidth="1"/>
-    <col min="39" max="40" width="20" customWidth="1"/>
-    <col min="41" max="41" width="30" customWidth="1"/>
-    <col min="42" max="42" width="20" customWidth="1"/>
-    <col min="43" max="43" width="15" customWidth="1"/>
-    <col min="44" max="44" width="30" customWidth="1"/>
-    <col min="45" max="49" width="15" customWidth="1"/>
-    <col min="50" max="50" width="30" customWidth="1"/>
-    <col min="51" max="51" width="15" customWidth="1"/>
-    <col min="52" max="53" width="20" customWidth="1"/>
-    <col min="54" max="54" width="30" customWidth="1"/>
-    <col min="55" max="55" width="20" customWidth="1"/>
-    <col min="56" max="57" width="15" customWidth="1"/>
-    <col min="58" max="59" width="20" customWidth="1"/>
-    <col min="60" max="61" width="15" customWidth="1"/>
-    <col min="62" max="63" width="20" customWidth="1"/>
-    <col min="64" max="65" width="15" customWidth="1"/>
-    <col min="66" max="67" width="20" customWidth="1"/>
-    <col min="68" max="69" width="15" customWidth="1"/>
-    <col min="70" max="71" width="20" customWidth="1"/>
-    <col min="72" max="72" width="15" customWidth="1"/>
-    <col min="73" max="76" width="20" customWidth="1"/>
-    <col min="77" max="77" width="15" customWidth="1"/>
-    <col min="78" max="81" width="20" customWidth="1"/>
-    <col min="82" max="83" width="15" customWidth="1"/>
-    <col min="84" max="87" width="20" customWidth="1"/>
-    <col min="88" max="89" width="15" customWidth="1"/>
-    <col min="90" max="93" width="20" customWidth="1"/>
-    <col min="94" max="95" width="15" customWidth="1"/>
-    <col min="96" max="99" width="20" customWidth="1"/>
-    <col min="100" max="101" width="15" customWidth="1"/>
-    <col min="102" max="105" width="20" customWidth="1"/>
-    <col min="106" max="107" width="15" customWidth="1"/>
-    <col min="108" max="114" width="20" customWidth="1"/>
-    <col min="115" max="115" width="15" customWidth="1"/>
-    <col min="116" max="119" width="20" customWidth="1"/>
-    <col min="120" max="120" width="15" customWidth="1"/>
-    <col min="121" max="128" width="20" customWidth="1"/>
-    <col min="129" max="129" width="30" customWidth="1"/>
-    <col min="130" max="131" width="15" customWidth="1"/>
-    <col min="132" max="133" width="10" customWidth="1"/>
-    <col min="134" max="134" width="20" customWidth="1"/>
-    <col min="135" max="135" width="15" customWidth="1"/>
-    <col min="136" max="136" width="20" customWidth="1"/>
-    <col min="137" max="138" width="15" customWidth="1"/>
-    <col min="139" max="143" width="20" customWidth="1"/>
-    <col min="144" max="147" width="30" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="14" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="25" customWidth="1"/>
+    <col min="17" max="17" width="17" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
+    <col min="19" max="19" width="17" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="19" customWidth="1"/>
+    <col min="22" max="22" width="17" customWidth="1"/>
+    <col min="23" max="23" width="21" customWidth="1"/>
+    <col min="24" max="25" width="25" customWidth="1"/>
+    <col min="26" max="27" width="14" customWidth="1"/>
+    <col min="28" max="28" width="18" customWidth="1"/>
+    <col min="29" max="31" width="14" customWidth="1"/>
+    <col min="32" max="32" width="17" customWidth="1"/>
+    <col min="33" max="33" width="22" customWidth="1"/>
+    <col min="34" max="34" width="18" customWidth="1"/>
+    <col min="35" max="35" width="25" customWidth="1"/>
+    <col min="36" max="36" width="29" customWidth="1"/>
+    <col min="37" max="37" width="15" customWidth="1"/>
+    <col min="38" max="38" width="16" customWidth="1"/>
+    <col min="39" max="39" width="23" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="42" width="16" customWidth="1"/>
+    <col min="43" max="43" width="21" customWidth="1"/>
+    <col min="44" max="44" width="25" customWidth="1"/>
+    <col min="45" max="45" width="19" customWidth="1"/>
+    <col min="46" max="46" width="21" customWidth="1"/>
+    <col min="47" max="47" width="19" customWidth="1"/>
+    <col min="48" max="48" width="17" customWidth="1"/>
+    <col min="49" max="49" width="26" customWidth="1"/>
+    <col min="50" max="50" width="23" customWidth="1"/>
+    <col min="51" max="51" width="26" customWidth="1"/>
+    <col min="52" max="52" width="32" customWidth="1"/>
+    <col min="53" max="53" width="22" customWidth="1"/>
+    <col min="54" max="54" width="23" customWidth="1"/>
+    <col min="55" max="55" width="15" customWidth="1"/>
+    <col min="56" max="57" width="24" customWidth="1"/>
+    <col min="58" max="58" width="21" customWidth="1"/>
+    <col min="59" max="59" width="15" customWidth="1"/>
+    <col min="60" max="61" width="24" customWidth="1"/>
+    <col min="62" max="62" width="21" customWidth="1"/>
+    <col min="63" max="63" width="15" customWidth="1"/>
+    <col min="64" max="65" width="24" customWidth="1"/>
+    <col min="66" max="66" width="21" customWidth="1"/>
+    <col min="67" max="67" width="15" customWidth="1"/>
+    <col min="68" max="69" width="24" customWidth="1"/>
+    <col min="70" max="70" width="21" customWidth="1"/>
+    <col min="71" max="71" width="22" customWidth="1"/>
+    <col min="72" max="72" width="31" customWidth="1"/>
+    <col min="73" max="73" width="37" customWidth="1"/>
+    <col min="74" max="74" width="27" customWidth="1"/>
+    <col min="75" max="75" width="28" customWidth="1"/>
+    <col min="76" max="76" width="20" customWidth="1"/>
+    <col min="77" max="77" width="29" customWidth="1"/>
+    <col min="78" max="78" width="35" customWidth="1"/>
+    <col min="79" max="79" width="25" customWidth="1"/>
+    <col min="80" max="81" width="26" customWidth="1"/>
+    <col min="82" max="83" width="35" customWidth="1"/>
+    <col min="84" max="84" width="40" customWidth="1"/>
+    <col min="85" max="85" width="31" customWidth="1"/>
+    <col min="86" max="86" width="32" customWidth="1"/>
+    <col min="87" max="87" width="26" customWidth="1"/>
+    <col min="88" max="89" width="35" customWidth="1"/>
+    <col min="90" max="90" width="40" customWidth="1"/>
+    <col min="91" max="91" width="31" customWidth="1"/>
+    <col min="92" max="92" width="32" customWidth="1"/>
+    <col min="93" max="93" width="26" customWidth="1"/>
+    <col min="94" max="95" width="35" customWidth="1"/>
+    <col min="96" max="96" width="40" customWidth="1"/>
+    <col min="97" max="97" width="31" customWidth="1"/>
+    <col min="98" max="98" width="32" customWidth="1"/>
+    <col min="99" max="99" width="26" customWidth="1"/>
+    <col min="100" max="101" width="35" customWidth="1"/>
+    <col min="102" max="102" width="40" customWidth="1"/>
+    <col min="103" max="103" width="31" customWidth="1"/>
+    <col min="104" max="104" width="32" customWidth="1"/>
+    <col min="105" max="105" width="26" customWidth="1"/>
+    <col min="106" max="107" width="35" customWidth="1"/>
+    <col min="108" max="108" width="40" customWidth="1"/>
+    <col min="109" max="109" width="31" customWidth="1"/>
+    <col min="110" max="110" width="32" customWidth="1"/>
+    <col min="111" max="111" width="21" customWidth="1"/>
+    <col min="112" max="112" width="14" customWidth="1"/>
+    <col min="113" max="113" width="15" customWidth="1"/>
+    <col min="114" max="114" width="21" customWidth="1"/>
+    <col min="115" max="115" width="30" customWidth="1"/>
+    <col min="116" max="116" width="36" customWidth="1"/>
+    <col min="117" max="117" width="26" customWidth="1"/>
+    <col min="118" max="118" width="27" customWidth="1"/>
+    <col min="119" max="119" width="19" customWidth="1"/>
+    <col min="120" max="120" width="28" customWidth="1"/>
+    <col min="121" max="121" width="34" customWidth="1"/>
+    <col min="122" max="122" width="24" customWidth="1"/>
+    <col min="123" max="123" width="25" customWidth="1"/>
+    <col min="124" max="124" width="29" customWidth="1"/>
+    <col min="125" max="126" width="14" customWidth="1"/>
+    <col min="127" max="127" width="25" customWidth="1"/>
+    <col min="128" max="128" width="29" customWidth="1"/>
+    <col min="129" max="129" width="27" customWidth="1"/>
+    <col min="130" max="131" width="30" customWidth="1"/>
+    <col min="132" max="132" width="17" customWidth="1"/>
+    <col min="133" max="133" width="15" customWidth="1"/>
+    <col min="134" max="134" width="21" customWidth="1"/>
+    <col min="135" max="135" width="18" customWidth="1"/>
+    <col min="136" max="136" width="22" customWidth="1"/>
+    <col min="137" max="137" width="21" customWidth="1"/>
+    <col min="138" max="138" width="17" customWidth="1"/>
+    <col min="139" max="139" width="24" customWidth="1"/>
+    <col min="140" max="141" width="16" customWidth="1"/>
+    <col min="142" max="142" width="19" customWidth="1"/>
+    <col min="143" max="144" width="14" customWidth="1"/>
+    <col min="145" max="145" width="19" customWidth="1"/>
+    <col min="146" max="146" width="20" customWidth="1"/>
+    <col min="147" max="147" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:147" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:147" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1222,156 +1259,155 @@
         <v>97</v>
       </c>
       <c r="CU1" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="CV1" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="CW1" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="CX1" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="CY1" s="1" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="CZ1" s="1" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="DA1" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="DB1" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="DC1" s="1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="DD1" s="1" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="DE1" s="1" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="DF1" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="DG1" s="1" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="DH1" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="DI1" s="1" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="DJ1" s="1" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="DK1" s="1" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="DL1" s="1" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="DM1" s="1" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="DN1" s="1" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="DO1" s="1" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="DP1" s="1" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="DQ1" s="1" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="DR1" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="DS1" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="DT1" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="DU1" s="1" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="DV1" s="1" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="DW1" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="DX1" s="1" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="DY1" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="DZ1" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="EA1" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="EB1" s="1" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="EC1" s="1" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="ED1" s="1" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="EE1" s="1" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="EF1" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="EG1" s="1" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="EH1" s="1" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="EI1" s="1" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="EJ1" s="1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="EK1" s="1" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="EL1" s="1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="EM1" s="1" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="EN1" s="1" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="EO1" s="1" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="EP1" s="1" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="EQ1" s="1" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>